<commit_message>
fix: Khắc phục triệt để lỗi lệch số liệu Quý 2 trên B04, B02, so lieu, Thue và Macro VBA
</commit_message>
<xml_diff>
--- a/output/Bao_Cao_Hop_Nhat_Q1_2026.xlsx
+++ b/output/Bao_Cao_Hop_Nhat_Q1_2026.xlsx
@@ -9394,7 +9394,7 @@
       </c>
       <c r="C8" s="705" t="inlineStr">
         <is>
-          <t>QUÝ 2 NĂM 2026</t>
+          <t>QUÝ 1 NĂM 2026</t>
         </is>
       </c>
     </row>
@@ -9561,10 +9561,10 @@
         </is>
       </c>
       <c r="C22" s="713" t="n">
-        <v>231464686791</v>
+        <v>443090394974</v>
       </c>
       <c r="D22" s="713" t="n">
-        <v>231464686791</v>
+        <v>443090394974</v>
       </c>
       <c r="E22" s="714" t="inlineStr">
         <is>
@@ -9584,10 +9584,10 @@
         </is>
       </c>
       <c r="C23" s="713" t="n">
-        <v>52142209214992</v>
+        <v>38955289723766</v>
       </c>
       <c r="D23" s="713" t="n">
-        <v>52142209214992</v>
+        <v>38955289723766</v>
       </c>
       <c r="E23" s="714" t="inlineStr">
         <is>
@@ -9607,10 +9607,10 @@
         </is>
       </c>
       <c r="C24" s="713" t="n">
-        <v>315725226474</v>
+        <v>226089518904</v>
       </c>
       <c r="D24" s="713" t="n">
-        <v>315725226474</v>
+        <v>226089518904</v>
       </c>
       <c r="E24" s="714" t="inlineStr">
         <is>
@@ -12314,8 +12314,9 @@
         </is>
       </c>
       <c r="C78" s="418" t="n"/>
-      <c r="D78" s="540" t="n">
-        <v>50000000000</v>
+      <c r="D78" s="540">
+        <f>'so lieu'!G36</f>
+        <v/>
       </c>
       <c r="E78" s="540" t="n">
         <v>50000000000</v>
@@ -12472,8 +12473,9 @@
         </is>
       </c>
       <c r="C84" s="418" t="n"/>
-      <c r="D84" s="540" t="n">
-        <v>9129514079</v>
+      <c r="D84" s="540">
+        <f>'so lieu'!G37+'so lieu'!G38</f>
+        <v/>
       </c>
       <c r="E84" s="540" t="n">
         <v>9129514079</v>
@@ -15931,8 +15933,9 @@
         </is>
       </c>
       <c r="C50" s="135" t="n"/>
-      <c r="D50" s="591" t="n">
-        <v>58000000000</v>
+      <c r="D50" s="591">
+        <f>'so lieu'!B3</f>
+        <v/>
       </c>
       <c r="E50" s="591" t="n">
         <v>72000000000</v>
@@ -17610,8 +17613,9 @@
         </is>
       </c>
       <c r="C112" s="115" t="n"/>
-      <c r="D112" s="585" t="n">
-        <v>512482745684</v>
+      <c r="D112" s="585">
+        <f>'so lieu'!B1+'so lieu'!B2+'so lieu'!B4</f>
+        <v/>
       </c>
       <c r="E112" s="585" t="n">
         <v>194465890088</v>
@@ -17649,7 +17653,10 @@
         </is>
       </c>
       <c r="C113" s="115" t="n"/>
-      <c r="D113" s="585" t="n"/>
+      <c r="D113" s="585">
+        <f>D114-D111-D112</f>
+        <v/>
+      </c>
       <c r="E113" s="585" t="n"/>
       <c r="F113" s="451" t="inlineStr">
         <is>
@@ -20650,8 +20657,9 @@
           <t>1. Thuế GTGT</t>
         </is>
       </c>
-      <c r="B199" s="656" t="n">
-        <v>327740170</v>
+      <c r="B199" s="656">
+        <f>Thue!D12</f>
+        <v/>
       </c>
       <c r="C199" s="656">
         <f>Thue!E12</f>
@@ -20696,8 +20704,9 @@
           <t>3. Thuế TNDN</t>
         </is>
       </c>
-      <c r="B202" s="656" t="n">
-        <v>1699375943</v>
+      <c r="B202" s="656">
+        <f>Thue!D16</f>
+        <v/>
       </c>
       <c r="C202" s="656">
         <f>Thue!E16</f>
@@ -21550,20 +21559,20 @@
         <v>2104207557</v>
       </c>
       <c r="E11" s="666" t="n">
-        <v>2247355787</v>
+        <v>2533921770</v>
       </c>
       <c r="F11" s="666" t="n">
-        <v>3229324778</v>
+        <v>3515890761</v>
       </c>
       <c r="G11" s="666" t="n">
-        <v>2247355787</v>
+        <v>2533921770</v>
       </c>
       <c r="H11" s="662" t="n"/>
       <c r="I11" s="662" t="n"/>
       <c r="J11" s="662" t="n"/>
       <c r="K11" s="661" t="n"/>
       <c r="L11" s="666" t="n">
-        <v>3229324778</v>
+        <v>3515890761</v>
       </c>
       <c r="M11" s="666" t="n">
         <v>1122238566</v>
@@ -21586,20 +21595,20 @@
         <v>327740170</v>
       </c>
       <c r="E12" s="667" t="n">
-        <v>929981117</v>
+        <v>1216547100</v>
       </c>
       <c r="F12" s="667" t="n">
-        <v>924519785</v>
+        <v>1211085768</v>
       </c>
       <c r="G12" s="667" t="n">
-        <v>929981117</v>
+        <v>1216547100</v>
       </c>
       <c r="H12" s="662" t="n"/>
       <c r="I12" s="662" t="n"/>
       <c r="J12" s="662" t="n"/>
       <c r="K12" s="661" t="n"/>
       <c r="L12" s="667" t="n">
-        <v>924519785</v>
+        <v>1211085768</v>
       </c>
       <c r="M12" s="667" t="n">
         <v>333201502</v>
@@ -22090,20 +22099,20 @@
         <v>2104207557</v>
       </c>
       <c r="E26" s="666" t="n">
-        <v>2247355787</v>
+        <v>2533921770</v>
       </c>
       <c r="F26" s="666" t="n">
-        <v>3229324778</v>
+        <v>3515890761</v>
       </c>
       <c r="G26" s="666" t="n">
-        <v>2247355787</v>
+        <v>2533921770</v>
       </c>
       <c r="H26" s="662" t="n"/>
       <c r="I26" s="662" t="n"/>
       <c r="J26" s="662" t="n"/>
       <c r="K26" s="661" t="n"/>
       <c r="L26" s="666" t="n">
-        <v>3229324778</v>
+        <v>3515890761</v>
       </c>
       <c r="M26" s="666" t="n">
         <v>1122238566</v>
@@ -30482,30 +30491,26 @@
       </c>
     </row>
     <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Chênh lệch (Nợ - Có)</t>
+        </is>
+      </c>
       <c r="B86" s="668">
-        <f>B85-[4]Sheet1!C65</f>
-        <v/>
-      </c>
-      <c r="C86" s="668">
-        <f>C85-[4]Sheet1!D65</f>
-        <v/>
-      </c>
+        <f>B85-C85</f>
+        <v/>
+      </c>
+      <c r="C86" s="668" t="n"/>
       <c r="D86" s="668">
-        <f>D85-[4]Sheet1!E65</f>
-        <v/>
-      </c>
-      <c r="E86" s="668">
-        <f>E85-[4]Sheet1!F65</f>
-        <v/>
-      </c>
+        <f>D85-E85</f>
+        <v/>
+      </c>
+      <c r="E86" s="668" t="n"/>
       <c r="F86" s="668">
-        <f>F85-[4]Sheet1!G65</f>
-        <v/>
-      </c>
-      <c r="G86" s="668">
-        <f>G85-[4]Sheet1!H65</f>
-        <v/>
-      </c>
+        <f>F85-G85</f>
+        <v/>
+      </c>
+      <c r="G86" s="668" t="n"/>
       <c r="J86" s="674" t="n"/>
       <c r="K86" s="274" t="n">
         <v>185339361569</v>

</xml_diff>